<commit_message>
Ask each creator how they work with drinks brands on TikTok
Ethan and Lauren already post gin and bottomless-brunch venues on TikTok,
so they may know the approval route better than we do. The email and DM now
ask whether a creator posts TikTok collaborations, has worked with an
alcohol brand there, and is set up on TikTok One, and the outreach tracker
has a column for the answer.

It is fact-finding only. The collaboration stays on Instagram until Tap That
has TikTok approval, and the internal plan says to decline any offer to post
without #ad or without a tag.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YQfykwfNBEN7oj3dqQfufW
</commit_message>
<xml_diff>
--- a/02 Design/02 Working Drafts/79__Influencer-Tracker__Tap-That-Brewery__Internal__Draft__v01.xlsx
+++ b/02 Design/02 Working Drafts/79__Influencer-Tracker__Tap-That-Brewery__Internal__Draft__v01.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Shortlist'!$A$4:$N$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Top 10'!$A$4:$F$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach Tracker'!$A$4:$P$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Outreach Tracker'!$A$4:$Q$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Content &amp; Results'!$A$4:$W$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Compliance Checklist'!$A$4:$D$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Partner Channels'!$A$4:$C$6</definedName>
@@ -101,9 +101,7 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2769,7 +2767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2787,7 +2785,8 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2804,6 +2803,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2881,6 +2881,11 @@
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>TikTok answer (on TikTok One? alcohol collabs before?)</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2920,7 +2925,8 @@
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr"/>
       <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -2956,7 +2962,8 @@
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
-      <c r="P6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -2992,7 +2999,8 @@
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="4" t="inlineStr"/>
       <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -3028,7 +3036,8 @@
       <c r="M8" s="5" t="inlineStr"/>
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -3064,7 +3073,8 @@
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -3100,7 +3110,8 @@
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -3136,7 +3147,8 @@
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="n"/>
+      <c r="Q11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -3172,7 +3184,8 @@
       <c r="M12" s="5" t="inlineStr"/>
       <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr"/>
-      <c r="P12" s="5" t="inlineStr"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -3208,7 +3221,8 @@
       <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="n"/>
+      <c r="Q13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -3244,7 +3258,8 @@
       <c r="M14" s="5" t="inlineStr"/>
       <c r="N14" s="5" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr"/>
-      <c r="P14" s="5" t="inlineStr"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -3280,7 +3295,8 @@
       <c r="M15" s="4" t="inlineStr"/>
       <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="n"/>
+      <c r="Q15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -3316,7 +3332,8 @@
       <c r="M16" s="5" t="inlineStr"/>
       <c r="N16" s="5" t="inlineStr"/>
       <c r="O16" s="5" t="inlineStr"/>
-      <c r="P16" s="5" t="inlineStr"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -3352,7 +3369,8 @@
       <c r="M17" s="4" t="inlineStr"/>
       <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -3388,7 +3406,8 @@
       <c r="M18" s="5" t="inlineStr"/>
       <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr"/>
-      <c r="P18" s="5" t="inlineStr"/>
+      <c r="P18" s="5" t="n"/>
+      <c r="Q18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -3424,7 +3443,8 @@
       <c r="M19" s="4" t="inlineStr"/>
       <c r="N19" s="4" t="inlineStr"/>
       <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="n"/>
+      <c r="Q19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -3460,7 +3480,8 @@
       <c r="M20" s="5" t="inlineStr"/>
       <c r="N20" s="5" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr"/>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -3496,7 +3517,8 @@
       <c r="M21" s="4" t="inlineStr"/>
       <c r="N21" s="4" t="inlineStr"/>
       <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -3532,7 +3554,8 @@
       <c r="M22" s="5" t="inlineStr"/>
       <c r="N22" s="5" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr"/>
-      <c r="P22" s="5" t="inlineStr"/>
+      <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -3568,7 +3591,8 @@
       <c r="M23" s="4" t="inlineStr"/>
       <c r="N23" s="4" t="inlineStr"/>
       <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="n"/>
+      <c r="Q23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -3604,7 +3628,8 @@
       <c r="M24" s="5" t="inlineStr"/>
       <c r="N24" s="5" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr"/>
-      <c r="P24" s="5" t="inlineStr"/>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -3640,7 +3665,8 @@
       <c r="M25" s="4" t="inlineStr"/>
       <c r="N25" s="4" t="inlineStr"/>
       <c r="O25" s="4" t="inlineStr"/>
-      <c r="P25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="n"/>
+      <c r="Q25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -3676,7 +3702,8 @@
       <c r="M26" s="5" t="inlineStr"/>
       <c r="N26" s="5" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr"/>
-      <c r="P26" s="5" t="inlineStr"/>
+      <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -3712,7 +3739,8 @@
       <c r="M27" s="4" t="inlineStr"/>
       <c r="N27" s="4" t="inlineStr"/>
       <c r="O27" s="4" t="inlineStr"/>
-      <c r="P27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="n"/>
+      <c r="Q27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -3748,7 +3776,8 @@
       <c r="M28" s="5" t="inlineStr"/>
       <c r="N28" s="5" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
-      <c r="P28" s="5" t="inlineStr"/>
+      <c r="P28" s="5" t="n"/>
+      <c r="Q28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -3784,7 +3813,8 @@
       <c r="M29" s="4" t="inlineStr"/>
       <c r="N29" s="4" t="inlineStr"/>
       <c r="O29" s="4" t="inlineStr"/>
-      <c r="P29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="n"/>
+      <c r="Q29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -3820,7 +3850,8 @@
       <c r="M30" s="5" t="inlineStr"/>
       <c r="N30" s="5" t="inlineStr"/>
       <c r="O30" s="5" t="inlineStr"/>
-      <c r="P30" s="5" t="inlineStr"/>
+      <c r="P30" s="5" t="n"/>
+      <c r="Q30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3856,10 +3887,11 @@
       <c r="M31" s="4" t="inlineStr"/>
       <c r="N31" s="4" t="inlineStr"/>
       <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="n"/>
+      <c r="Q31" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:P31"/>
+  <autoFilter ref="A4:Q31"/>
   <dataValidations count="4">
     <dataValidation sqref="E5:E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>

</xml_diff>